<commit_message>
Se agregan tablas principales
</commit_message>
<xml_diff>
--- a/Tablas.xlsx
+++ b/Tablas.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Carrera-Historial" sheetId="1" state="visible" r:id="rId3"/>
@@ -15,6 +15,7 @@
     <sheet name="Años" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Niveles" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Horarios" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Inscripcion" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="181">
   <si>
     <t xml:space="preserve">major</t>
   </si>
@@ -563,6 +564,12 @@
   </si>
   <si>
     <t xml:space="preserve">Numero de Seccion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_profesor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_folio</t>
   </si>
 </sst>
 </file>
@@ -670,7 +677,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -715,8 +722,12 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -3353,7 +3364,9 @@
       <c r="H24" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="I24" s="11"/>
+      <c r="I24" s="11" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="n">
@@ -3379,6 +3392,9 @@
       </c>
       <c r="H25" s="9" t="n">
         <v>2000</v>
+      </c>
+      <c r="I25" s="12" t="n">
+        <v>4000</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3407,6 +3423,9 @@
       <c r="H26" s="9" t="n">
         <v>2001</v>
       </c>
+      <c r="I26" s="12" t="n">
+        <v>4001</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="n">
@@ -3434,6 +3453,9 @@
       <c r="H27" s="9" t="n">
         <v>2002</v>
       </c>
+      <c r="I27" s="12" t="n">
+        <v>4002</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="n">
@@ -3461,6 +3483,9 @@
       <c r="H28" s="9" t="n">
         <v>2002</v>
       </c>
+      <c r="I28" s="12" t="n">
+        <v>4003</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="n">
@@ -3488,6 +3513,9 @@
       <c r="H29" s="9" t="n">
         <v>2000</v>
       </c>
+      <c r="I29" s="12" t="n">
+        <v>4004</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="n">
@@ -3515,6 +3543,9 @@
       <c r="H30" s="9" t="n">
         <v>2001</v>
       </c>
+      <c r="I30" s="12" t="n">
+        <v>4005</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="n">
@@ -3542,6 +3573,9 @@
       <c r="H31" s="9" t="n">
         <v>2002</v>
       </c>
+      <c r="I31" s="12" t="n">
+        <v>4000</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="n">
@@ -3569,6 +3603,9 @@
       <c r="H32" s="9" t="n">
         <v>2001</v>
       </c>
+      <c r="I32" s="12" t="n">
+        <v>4006</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="n">
@@ -3596,6 +3633,9 @@
       <c r="H33" s="9" t="n">
         <v>2002</v>
       </c>
+      <c r="I33" s="12" t="n">
+        <v>4005</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="n">
@@ -3623,6 +3663,9 @@
       <c r="H34" s="9" t="n">
         <v>2000</v>
       </c>
+      <c r="I34" s="12" t="n">
+        <v>4007</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="n">
@@ -3650,6 +3693,9 @@
       <c r="H35" s="9" t="n">
         <v>2001</v>
       </c>
+      <c r="I35" s="12" t="n">
+        <v>4000</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="n">
@@ -3677,6 +3723,9 @@
       <c r="H36" s="9" t="n">
         <v>2000</v>
       </c>
+      <c r="I36" s="12" t="n">
+        <v>4005</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="n">
@@ -3704,6 +3753,9 @@
       <c r="H37" s="9" t="n">
         <v>2002</v>
       </c>
+      <c r="I37" s="12" t="n">
+        <v>4008</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="n">
@@ -3731,6 +3783,9 @@
       <c r="H38" s="9" t="n">
         <v>2000</v>
       </c>
+      <c r="I38" s="12" t="n">
+        <v>4005</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="n">
@@ -3758,6 +3813,9 @@
       <c r="H39" s="9" t="n">
         <v>2000</v>
       </c>
+      <c r="I39" s="12" t="n">
+        <v>4009</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="n">
@@ -3785,6 +3843,9 @@
       <c r="H40" s="9" t="n">
         <v>2001</v>
       </c>
+      <c r="I40" s="12" t="n">
+        <v>4000</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="n">
@@ -3812,6 +3873,9 @@
       <c r="H41" s="9" t="n">
         <v>2002</v>
       </c>
+      <c r="I41" s="12" t="n">
+        <v>4006</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="n">
@@ -3839,6 +3903,9 @@
       <c r="H42" s="9" t="n">
         <v>2001</v>
       </c>
+      <c r="I42" s="12" t="n">
+        <v>4010</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="n">
@@ -3865,6 +3932,9 @@
       </c>
       <c r="H43" s="9" t="n">
         <v>2000</v>
+      </c>
+      <c r="I43" s="12" t="n">
+        <v>4010</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4311,4 +4381,243 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="12" t="n">
+        <v>5000</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="12" t="n">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="12" t="n">
+        <v>5001</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="12" t="n">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="n">
+        <v>5002</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="12" t="n">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="n">
+        <v>5003</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="n">
+        <v>5004</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="n">
+        <v>5005</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="n">
+        <v>5006</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="n">
+        <v>5007</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="n">
+        <v>5008</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="n">
+        <v>5009</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="n">
+        <v>5010</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12" t="n">
+        <v>5011</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="12" t="n">
+        <v>5012</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12" t="n">
+        <v>5013</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12" t="n">
+        <v>5015</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="12" t="n">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="n">
+        <v>5016</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="12" t="n">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="n">
+        <v>5017</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="12" t="n">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12" t="n">
+        <v>5018</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="12" t="n">
+        <v>5019</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>519</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>